<commit_message>
Add site qmds, update quarto config and audit runner
Add per-site Quarto pages (Nairobi, Eldoret, Kisumu, Mombasa) and a new _quarto.yaml to configure the website navbar, theme, and output dir. Rename main analysis QMD to index.qmd, remove legacy _quarto.yml.txt, and add a Nairobi.txt artifact. Update R/run_audit.R to source reports/render_all_reports.R and continue discovering sites from data/raw. Also include updated Kisumu audit output (Excel) and diagram (PNG). These changes integrate site-specific reports into the website and ensure the audit runner pulls in the report rendering logic.
</commit_message>
<xml_diff>
--- a/data/audit_outputs/Kisumu_RDS_audit.xlsx
+++ b/data/audit_outputs/Kisumu_RDS_audit.xlsx
@@ -415,7 +415,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -423,7 +423,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>342</v>
+        <v>363</v>
       </c>
     </row>
     <row r="6">
@@ -431,7 +431,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>325</v>
+        <v>348</v>
       </c>
     </row>
     <row r="7">
@@ -439,7 +439,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -447,7 +447,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -455,7 +455,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>